<commit_message>
fix: Stock bajo basado en cajas (unBx * 10)
</commit_message>
<xml_diff>
--- a/frontend/public/reports/StockPulse_ESCOLAR.xlsx
+++ b/frontend/public/reports/StockPulse_ESCOLAR.xlsx
@@ -7242,11 +7242,11 @@
       <c r="E11">
         <v>96</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="6">
         <v>31</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>10</v>
+      <c r="G11" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -7265,11 +7265,11 @@
       <c r="E12">
         <v>96</v>
       </c>
-      <c r="F12" s="2">
-        <v>10</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>10</v>
+      <c r="F12" s="6">
+        <v>10</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -7403,11 +7403,11 @@
       <c r="E18">
         <v>288</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="6">
         <v>854</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>10</v>
+      <c r="G18" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -7518,11 +7518,11 @@
       <c r="E23">
         <v>300</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="6">
         <v>1775</v>
       </c>
-      <c r="G23" s="3" t="s">
-        <v>10</v>
+      <c r="G23" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -8044,11 +8044,11 @@
       <c r="E14">
         <v>50</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="6">
         <v>471</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>10</v>
+      <c r="G14" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -8067,11 +8067,11 @@
       <c r="E15">
         <v>50</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="6">
         <v>445</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>10</v>
+      <c r="G15" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -8251,11 +8251,11 @@
       <c r="E23">
         <v>50</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="6">
         <v>14</v>
       </c>
-      <c r="G23" s="3" t="s">
-        <v>10</v>
+      <c r="G23" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -8826,11 +8826,11 @@
       <c r="E48">
         <v>100</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="6">
         <v>42</v>
       </c>
-      <c r="G48" s="3" t="s">
-        <v>10</v>
+      <c r="G48" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -8964,11 +8964,11 @@
       <c r="E54">
         <v>100</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="6">
         <v>751</v>
       </c>
-      <c r="G54" s="3" t="s">
-        <v>10</v>
+      <c r="G54" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -9102,11 +9102,11 @@
       <c r="E60">
         <v>100</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="6">
         <v>645</v>
       </c>
-      <c r="G60" s="3" t="s">
-        <v>10</v>
+      <c r="G60" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
@@ -9194,11 +9194,11 @@
       <c r="E64">
         <v>100</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="6">
         <v>253</v>
       </c>
-      <c r="G64" s="3" t="s">
-        <v>10</v>
+      <c r="G64" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
@@ -9355,11 +9355,11 @@
       <c r="E71">
         <v>100</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="6">
         <v>100</v>
       </c>
-      <c r="G71" s="3" t="s">
-        <v>10</v>
+      <c r="G71" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
@@ -9677,11 +9677,11 @@
       <c r="E85">
         <v>100</v>
       </c>
-      <c r="F85" s="2">
+      <c r="F85" s="6">
         <v>13</v>
       </c>
-      <c r="G85" s="3" t="s">
-        <v>10</v>
+      <c r="G85" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
@@ -9838,11 +9838,11 @@
       <c r="E92">
         <v>100</v>
       </c>
-      <c r="F92" s="2">
+      <c r="F92" s="6">
         <v>940</v>
       </c>
-      <c r="G92" s="3" t="s">
-        <v>10</v>
+      <c r="G92" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
@@ -9976,11 +9976,11 @@
       <c r="E98">
         <v>120</v>
       </c>
-      <c r="F98" s="2">
+      <c r="F98" s="6">
         <v>26</v>
       </c>
-      <c r="G98" s="3" t="s">
-        <v>10</v>
+      <c r="G98" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
@@ -10068,11 +10068,11 @@
       <c r="E102">
         <v>120</v>
       </c>
-      <c r="F102" s="2">
+      <c r="F102" s="6">
         <v>60</v>
       </c>
-      <c r="G102" s="3" t="s">
-        <v>10</v>
+      <c r="G102" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
@@ -10091,11 +10091,11 @@
       <c r="E103">
         <v>120</v>
       </c>
-      <c r="F103" s="2">
+      <c r="F103" s="6">
         <v>335</v>
       </c>
-      <c r="G103" s="3" t="s">
-        <v>10</v>
+      <c r="G103" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
@@ -10344,11 +10344,11 @@
       <c r="E114">
         <v>24</v>
       </c>
-      <c r="F114" s="2">
+      <c r="F114" s="6">
         <v>137</v>
       </c>
-      <c r="G114" s="3" t="s">
-        <v>10</v>
+      <c r="G114" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
@@ -10643,11 +10643,11 @@
       <c r="E127">
         <v>24</v>
       </c>
-      <c r="F127" s="2">
+      <c r="F127" s="6">
         <v>57</v>
       </c>
-      <c r="G127" s="3" t="s">
-        <v>10</v>
+      <c r="G127" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.25">
@@ -10919,11 +10919,11 @@
       <c r="E139">
         <v>30</v>
       </c>
-      <c r="F139" s="2">
+      <c r="F139" s="6">
         <v>49</v>
       </c>
-      <c r="G139" s="3" t="s">
-        <v>10</v>
+      <c r="G139" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
@@ -10942,11 +10942,11 @@
       <c r="E140">
         <v>30</v>
       </c>
-      <c r="F140" s="2">
+      <c r="F140" s="6">
         <v>297</v>
       </c>
-      <c r="G140" s="3" t="s">
-        <v>10</v>
+      <c r="G140" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
@@ -10965,11 +10965,11 @@
       <c r="E141">
         <v>30</v>
       </c>
-      <c r="F141" s="2">
+      <c r="F141" s="6">
         <v>180</v>
       </c>
-      <c r="G141" s="3" t="s">
-        <v>10</v>
+      <c r="G141" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
@@ -11356,11 +11356,11 @@
       <c r="E158">
         <v>24</v>
       </c>
-      <c r="F158" s="2">
+      <c r="F158" s="6">
         <v>17</v>
       </c>
-      <c r="G158" s="3" t="s">
-        <v>10</v>
+      <c r="G158" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
@@ -11379,11 +11379,11 @@
       <c r="E159">
         <v>24</v>
       </c>
-      <c r="F159" s="2">
+      <c r="F159" s="6">
         <v>130</v>
       </c>
-      <c r="G159" s="3" t="s">
-        <v>10</v>
+      <c r="G159" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.25">
@@ -11770,11 +11770,11 @@
       <c r="E176">
         <v>48</v>
       </c>
-      <c r="F176" s="2">
+      <c r="F176" s="6">
         <v>48</v>
       </c>
-      <c r="G176" s="3" t="s">
-        <v>10</v>
+      <c r="G176" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.25">
@@ -11793,11 +11793,11 @@
       <c r="E177">
         <v>48</v>
       </c>
-      <c r="F177" s="2">
+      <c r="F177" s="6">
         <v>193</v>
       </c>
-      <c r="G177" s="3" t="s">
-        <v>10</v>
+      <c r="G177" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.25">
@@ -11839,11 +11839,11 @@
       <c r="E179">
         <v>36</v>
       </c>
-      <c r="F179" s="2">
+      <c r="F179" s="6">
         <v>218</v>
       </c>
-      <c r="G179" s="3" t="s">
-        <v>10</v>
+      <c r="G179" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="180" spans="1:7" x14ac:dyDescent="0.25">
@@ -11977,11 +11977,11 @@
       <c r="E185">
         <v>240</v>
       </c>
-      <c r="F185" s="2">
+      <c r="F185" s="6">
         <v>1086</v>
       </c>
-      <c r="G185" s="3" t="s">
-        <v>10</v>
+      <c r="G185" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.25">
@@ -12299,11 +12299,11 @@
       <c r="E199">
         <v>10</v>
       </c>
-      <c r="F199" s="2">
+      <c r="F199" s="6">
         <v>69</v>
       </c>
-      <c r="G199" s="3" t="s">
-        <v>10</v>
+      <c r="G199" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.25">
@@ -12437,11 +12437,11 @@
       <c r="E205">
         <v>280</v>
       </c>
-      <c r="F205" s="2">
+      <c r="F205" s="6">
         <v>745</v>
       </c>
-      <c r="G205" s="3" t="s">
-        <v>10</v>
+      <c r="G205" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.25">
@@ -12506,11 +12506,11 @@
       <c r="E208">
         <v>720</v>
       </c>
-      <c r="F208" s="2">
+      <c r="F208" s="6">
         <v>5462</v>
       </c>
-      <c r="G208" s="3" t="s">
-        <v>10</v>
+      <c r="G208" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.25">
@@ -12529,11 +12529,11 @@
       <c r="E209">
         <v>720</v>
       </c>
-      <c r="F209" s="2">
+      <c r="F209" s="6">
         <v>6036</v>
       </c>
-      <c r="G209" s="3" t="s">
-        <v>10</v>
+      <c r="G209" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.25">
@@ -12575,11 +12575,11 @@
       <c r="E211">
         <v>720</v>
       </c>
-      <c r="F211" s="2">
+      <c r="F211" s="6">
         <v>848</v>
       </c>
-      <c r="G211" s="3" t="s">
-        <v>10</v>
+      <c r="G211" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="212" spans="1:7" x14ac:dyDescent="0.25">
@@ -12598,11 +12598,11 @@
       <c r="E212">
         <v>720</v>
       </c>
-      <c r="F212" s="2">
+      <c r="F212" s="6">
         <v>4603</v>
       </c>
-      <c r="G212" s="3" t="s">
-        <v>10</v>
+      <c r="G212" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.25">
@@ -12621,11 +12621,11 @@
       <c r="E213">
         <v>720</v>
       </c>
-      <c r="F213" s="2">
+      <c r="F213" s="6">
         <v>369</v>
       </c>
-      <c r="G213" s="3" t="s">
-        <v>10</v>
+      <c r="G213" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.25">
@@ -12644,11 +12644,11 @@
       <c r="E214">
         <v>720</v>
       </c>
-      <c r="F214" s="2">
+      <c r="F214" s="6">
         <v>3947</v>
       </c>
-      <c r="G214" s="3" t="s">
-        <v>10</v>
+      <c r="G214" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.25">
@@ -13817,11 +13817,11 @@
       <c r="E265">
         <v>5</v>
       </c>
-      <c r="F265" s="2">
+      <c r="F265" s="6">
         <v>27</v>
       </c>
-      <c r="G265" s="3" t="s">
-        <v>10</v>
+      <c r="G265" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.25">
@@ -13840,11 +13840,11 @@
       <c r="E266">
         <v>5</v>
       </c>
-      <c r="F266" s="2">
+      <c r="F266" s="6">
         <v>26</v>
       </c>
-      <c r="G266" s="3" t="s">
-        <v>10</v>
+      <c r="G266" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -13998,11 +13998,11 @@
       <c r="E6">
         <v>18</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="6">
         <v>115</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>10</v>
+      <c r="G6" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -14665,11 +14665,11 @@
       <c r="E35">
         <v>576</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="6">
         <v>2304</v>
       </c>
-      <c r="G35" s="3" t="s">
-        <v>10</v>
+      <c r="G35" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -14711,11 +14711,11 @@
       <c r="E37">
         <v>576</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="6">
         <v>1469</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>10</v>
+      <c r="G37" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -14734,11 +14734,11 @@
       <c r="E38">
         <v>576</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="6">
         <v>63</v>
       </c>
-      <c r="G38" s="3" t="s">
-        <v>10</v>
+      <c r="G38" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -14803,11 +14803,11 @@
       <c r="E41">
         <v>576</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="6">
         <v>2846</v>
       </c>
-      <c r="G41" s="3" t="s">
-        <v>10</v>
+      <c r="G41" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -14826,11 +14826,11 @@
       <c r="E42">
         <v>576</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="6">
         <v>981</v>
       </c>
-      <c r="G42" s="3" t="s">
-        <v>10</v>
+      <c r="G42" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -14872,11 +14872,11 @@
       <c r="E44">
         <v>576</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="6">
         <v>125</v>
       </c>
-      <c r="G44" s="3" t="s">
-        <v>10</v>
+      <c r="G44" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -15766,11 +15766,11 @@
       <c r="E5">
         <v>288</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="6">
         <v>1038</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>10</v>
+      <c r="G5" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -16157,11 +16157,11 @@
       <c r="E22">
         <v>192</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="6">
         <v>1033</v>
       </c>
-      <c r="G22" s="3" t="s">
-        <v>10</v>
+      <c r="G22" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -16295,11 +16295,11 @@
       <c r="E28">
         <v>192</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="6">
         <v>122</v>
       </c>
-      <c r="G28" s="3" t="s">
-        <v>10</v>
+      <c r="G28" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -16410,11 +16410,11 @@
       <c r="E33">
         <v>144</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="6">
         <v>1001</v>
       </c>
-      <c r="G33" s="3" t="s">
-        <v>10</v>
+      <c r="G33" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -16456,11 +16456,11 @@
       <c r="E35">
         <v>144</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="6">
         <v>258</v>
       </c>
-      <c r="G35" s="3" t="s">
-        <v>10</v>
+      <c r="G35" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -16479,11 +16479,11 @@
       <c r="E36">
         <v>72</v>
       </c>
-      <c r="F36" s="2">
+      <c r="F36" s="6">
         <v>42</v>
       </c>
-      <c r="G36" s="3" t="s">
-        <v>10</v>
+      <c r="G36" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -16502,11 +16502,11 @@
       <c r="E37">
         <v>144</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="6">
         <v>344</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>10</v>
+      <c r="G37" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -16525,11 +16525,11 @@
       <c r="E38">
         <v>72</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="6">
         <v>235</v>
       </c>
-      <c r="G38" s="3" t="s">
-        <v>10</v>
+      <c r="G38" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -16548,11 +16548,11 @@
       <c r="E39">
         <v>144</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F39" s="6">
         <v>1014</v>
       </c>
-      <c r="G39" s="3" t="s">
-        <v>10</v>
+      <c r="G39" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -16571,11 +16571,11 @@
       <c r="E40">
         <v>72</v>
       </c>
-      <c r="F40" s="2">
+      <c r="F40" s="6">
         <v>120</v>
       </c>
-      <c r="G40" s="3" t="s">
-        <v>10</v>
+      <c r="G40" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -16594,11 +16594,11 @@
       <c r="E41">
         <v>144</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="6">
         <v>454</v>
       </c>
-      <c r="G41" s="3" t="s">
-        <v>10</v>
+      <c r="G41" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -16617,11 +16617,11 @@
       <c r="E42">
         <v>72</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="6">
         <v>60</v>
       </c>
-      <c r="G42" s="3" t="s">
-        <v>10</v>
+      <c r="G42" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -16640,11 +16640,11 @@
       <c r="E43">
         <v>144</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="6">
         <v>400</v>
       </c>
-      <c r="G43" s="3" t="s">
-        <v>10</v>
+      <c r="G43" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -16686,11 +16686,11 @@
       <c r="E45">
         <v>144</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="6">
         <v>273</v>
       </c>
-      <c r="G45" s="3" t="s">
-        <v>10</v>
+      <c r="G45" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -16732,11 +16732,11 @@
       <c r="E47">
         <v>144</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="6">
         <v>1400</v>
       </c>
-      <c r="G47" s="3" t="s">
-        <v>10</v>
+      <c r="G47" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -17215,11 +17215,11 @@
       <c r="E68">
         <v>200</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="6">
         <v>44</v>
       </c>
-      <c r="G68" s="3" t="s">
-        <v>10</v>
+      <c r="G68" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
@@ -17284,11 +17284,11 @@
       <c r="E71">
         <v>200</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="6">
         <v>1246</v>
       </c>
-      <c r="G71" s="3" t="s">
-        <v>10</v>
+      <c r="G71" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
@@ -17353,11 +17353,11 @@
       <c r="E74">
         <v>200</v>
       </c>
-      <c r="F74" s="2">
+      <c r="F74" s="6">
         <v>932</v>
       </c>
-      <c r="G74" s="3" t="s">
-        <v>10</v>
+      <c r="G74" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
@@ -17468,11 +17468,11 @@
       <c r="E79">
         <v>200</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="6">
         <v>1865</v>
       </c>
-      <c r="G79" s="3" t="s">
-        <v>10</v>
+      <c r="G79" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
@@ -17560,11 +17560,11 @@
       <c r="E83">
         <v>1152</v>
       </c>
-      <c r="F83" s="2">
+      <c r="F83" s="6">
         <v>227</v>
       </c>
-      <c r="G83" s="3" t="s">
-        <v>10</v>
+      <c r="G83" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
@@ -17606,11 +17606,11 @@
       <c r="E85">
         <v>1152</v>
       </c>
-      <c r="F85" s="2">
+      <c r="F85" s="6">
         <v>3385</v>
       </c>
-      <c r="G85" s="3" t="s">
-        <v>10</v>
+      <c r="G85" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
@@ -17652,11 +17652,11 @@
       <c r="E87">
         <v>576</v>
       </c>
-      <c r="F87" s="2">
+      <c r="F87" s="6">
         <v>4143</v>
       </c>
-      <c r="G87" s="3" t="s">
-        <v>10</v>
+      <c r="G87" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
@@ -17675,11 +17675,11 @@
       <c r="E88">
         <v>576</v>
       </c>
-      <c r="F88" s="2">
+      <c r="F88" s="6">
         <v>5653</v>
       </c>
-      <c r="G88" s="3" t="s">
-        <v>10</v>
+      <c r="G88" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -17698,11 +17698,11 @@
       <c r="E89">
         <v>576</v>
       </c>
-      <c r="F89" s="2">
+      <c r="F89" s="6">
         <v>207</v>
       </c>
-      <c r="G89" s="3" t="s">
-        <v>10</v>
+      <c r="G89" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
@@ -17721,11 +17721,11 @@
       <c r="E90">
         <v>576</v>
       </c>
-      <c r="F90" s="2">
+      <c r="F90" s="6">
         <v>1132</v>
       </c>
-      <c r="G90" s="3" t="s">
-        <v>10</v>
+      <c r="G90" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
@@ -17767,11 +17767,11 @@
       <c r="E92">
         <v>576</v>
       </c>
-      <c r="F92" s="2">
+      <c r="F92" s="6">
         <v>5395</v>
       </c>
-      <c r="G92" s="3" t="s">
-        <v>10</v>
+      <c r="G92" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
@@ -17905,11 +17905,11 @@
       <c r="E98">
         <v>144</v>
       </c>
-      <c r="F98" s="2">
+      <c r="F98" s="6">
         <v>233</v>
       </c>
-      <c r="G98" s="3" t="s">
-        <v>10</v>
+      <c r="G98" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
@@ -18181,11 +18181,11 @@
       <c r="E110">
         <v>192</v>
       </c>
-      <c r="F110" s="2">
+      <c r="F110" s="6">
         <v>1359</v>
       </c>
-      <c r="G110" s="3" t="s">
-        <v>10</v>
+      <c r="G110" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
@@ -18342,11 +18342,11 @@
       <c r="E117">
         <v>192</v>
       </c>
-      <c r="F117" s="2">
+      <c r="F117" s="6">
         <v>65</v>
       </c>
-      <c r="G117" s="3" t="s">
-        <v>10</v>
+      <c r="G117" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
@@ -18411,11 +18411,11 @@
       <c r="E120">
         <v>192</v>
       </c>
-      <c r="F120" s="2">
+      <c r="F120" s="6">
         <v>788</v>
       </c>
-      <c r="G120" s="3" t="s">
-        <v>10</v>
+      <c r="G120" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -18434,11 +18434,11 @@
       <c r="E121">
         <v>192</v>
       </c>
-      <c r="F121" s="2">
+      <c r="F121" s="6">
         <v>137</v>
       </c>
-      <c r="G121" s="3" t="s">
-        <v>10</v>
+      <c r="G121" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
@@ -18664,11 +18664,11 @@
       <c r="E131">
         <v>192</v>
       </c>
-      <c r="F131" s="2">
+      <c r="F131" s="6">
         <v>287</v>
       </c>
-      <c r="G131" s="3" t="s">
-        <v>10</v>
+      <c r="G131" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
@@ -18710,11 +18710,11 @@
       <c r="E133">
         <v>192</v>
       </c>
-      <c r="F133" s="2">
+      <c r="F133" s="6">
         <v>185</v>
       </c>
-      <c r="G133" s="3" t="s">
-        <v>10</v>
+      <c r="G133" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
@@ -18802,11 +18802,11 @@
       <c r="E137">
         <v>192</v>
       </c>
-      <c r="F137" s="2">
+      <c r="F137" s="6">
         <v>108</v>
       </c>
-      <c r="G137" s="3" t="s">
-        <v>10</v>
+      <c r="G137" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
@@ -18825,11 +18825,11 @@
       <c r="E138">
         <v>192</v>
       </c>
-      <c r="F138" s="2">
+      <c r="F138" s="6">
         <v>99</v>
       </c>
-      <c r="G138" s="3" t="s">
-        <v>10</v>
+      <c r="G138" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
@@ -18848,11 +18848,11 @@
       <c r="E139">
         <v>192</v>
       </c>
-      <c r="F139" s="2">
+      <c r="F139" s="6">
         <v>125</v>
       </c>
-      <c r="G139" s="3" t="s">
-        <v>10</v>
+      <c r="G139" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
@@ -18871,11 +18871,11 @@
       <c r="E140">
         <v>192</v>
       </c>
-      <c r="F140" s="2">
+      <c r="F140" s="6">
         <v>17</v>
       </c>
-      <c r="G140" s="3" t="s">
-        <v>10</v>
+      <c r="G140" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
@@ -18894,11 +18894,11 @@
       <c r="E141">
         <v>192</v>
       </c>
-      <c r="F141" s="2">
+      <c r="F141" s="6">
         <v>114</v>
       </c>
-      <c r="G141" s="3" t="s">
-        <v>10</v>
+      <c r="G141" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
@@ -18917,11 +18917,11 @@
       <c r="E142">
         <v>192</v>
       </c>
-      <c r="F142" s="2">
+      <c r="F142" s="6">
         <v>126</v>
       </c>
-      <c r="G142" s="3" t="s">
-        <v>10</v>
+      <c r="G142" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.25">
@@ -18940,11 +18940,11 @@
       <c r="E143">
         <v>192</v>
       </c>
-      <c r="F143" s="2">
+      <c r="F143" s="6">
         <v>42</v>
       </c>
-      <c r="G143" s="3" t="s">
-        <v>10</v>
+      <c r="G143" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
@@ -18963,11 +18963,11 @@
       <c r="E144">
         <v>192</v>
       </c>
-      <c r="F144" s="2">
+      <c r="F144" s="6">
         <v>58</v>
       </c>
-      <c r="G144" s="3" t="s">
-        <v>10</v>
+      <c r="G144" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -19788,11 +19788,11 @@
       <c r="E35">
         <v>120</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="6">
         <v>568</v>
       </c>
-      <c r="G35" s="3" t="s">
-        <v>10</v>
+      <c r="G35" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -20271,11 +20271,11 @@
       <c r="E56">
         <v>144</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="6">
         <v>19</v>
       </c>
-      <c r="G56" s="3" t="s">
-        <v>10</v>
+      <c r="G56" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -20593,11 +20593,11 @@
       <c r="E70">
         <v>12</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="6">
         <v>22</v>
       </c>
-      <c r="G70" s="3" t="s">
-        <v>10</v>
+      <c r="G70" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
@@ -20777,11 +20777,11 @@
       <c r="E78">
         <v>144</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="6">
         <v>936</v>
       </c>
-      <c r="G78" s="3" t="s">
-        <v>10</v>
+      <c r="G78" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
@@ -20800,11 +20800,11 @@
       <c r="E79">
         <v>144</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="6">
         <v>359</v>
       </c>
-      <c r="G79" s="3" t="s">
-        <v>10</v>
+      <c r="G79" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
@@ -20846,11 +20846,11 @@
       <c r="E81">
         <v>144</v>
       </c>
-      <c r="F81" s="2">
+      <c r="F81" s="6">
         <v>319</v>
       </c>
-      <c r="G81" s="3" t="s">
-        <v>10</v>
+      <c r="G81" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -20984,11 +20984,11 @@
       <c r="E87">
         <v>144</v>
       </c>
-      <c r="F87" s="2">
+      <c r="F87" s="6">
         <v>808</v>
       </c>
-      <c r="G87" s="3" t="s">
-        <v>10</v>
+      <c r="G87" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
@@ -21944,11 +21944,11 @@
       <c r="E26">
         <v>24</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="6">
         <v>202</v>
       </c>
-      <c r="G26" s="3" t="s">
-        <v>10</v>
+      <c r="G26" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -21967,11 +21967,11 @@
       <c r="E27">
         <v>24</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="6">
         <v>198</v>
       </c>
-      <c r="G27" s="3" t="s">
-        <v>10</v>
+      <c r="G27" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -22674,11 +22674,11 @@
       <c r="E2">
         <v>1000</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="6">
         <v>3238</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>10</v>
+      <c r="G2" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -22720,11 +22720,11 @@
       <c r="E4">
         <v>1000</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="6">
         <v>4021</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>10</v>
+      <c r="G4" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -22766,11 +22766,11 @@
       <c r="E6">
         <v>500</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="6">
         <v>207</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>10</v>
+      <c r="G6" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -22950,11 +22950,11 @@
       <c r="E14">
         <v>200</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="6">
         <v>1904</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>10</v>
+      <c r="G14" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -22973,11 +22973,11 @@
       <c r="E15">
         <v>120</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="6">
         <v>1063</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>10</v>
+      <c r="G15" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: script simplificado para Excel profesional
</commit_message>
<xml_diff>
--- a/frontend/public/reports/StockPulse_ESCOLAR.xlsx
+++ b/frontend/public/reports/StockPulse_ESCOLAR.xlsx
@@ -6219,6 +6219,7 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -6786,7 +6787,7 @@
         <v>25</v>
       </c>
       <c r="F6" s="2">
-        <v>3627</v>
+        <v>3927</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>10</v>
@@ -6924,7 +6925,7 @@
         <v>25</v>
       </c>
       <c r="F12" s="2">
-        <v>25453</v>
+        <v>25578</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>10</v>
@@ -14965,7 +14966,7 @@
         <v>144</v>
       </c>
       <c r="F48" s="2">
-        <v>49096</v>
+        <v>49384</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>10</v>
@@ -19927,7 +19928,7 @@
         <v>144</v>
       </c>
       <c r="F41" s="2">
-        <v>7758</v>
+        <v>7902</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>10</v>
@@ -21393,7 +21394,7 @@
         <v>12</v>
       </c>
       <c r="F2" s="2">
-        <v>1172</v>
+        <v>1184</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>10</v>
@@ -21462,7 +21463,7 @@
         <v>12</v>
       </c>
       <c r="F5" s="2">
-        <v>862</v>
+        <v>874</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>10</v>

</xml_diff>